<commit_message>
Rebalance Forever Bambu personnel costs
</commit_message>
<xml_diff>
--- a/forever-bambu/allegati/Allegato_B_Forever_Bambu_compilato.xlsx
+++ b/forever-bambu/allegati/Allegato_B_Forever_Bambu_compilato.xlsx
@@ -1713,10 +1713,8 @@
       <c r="B6" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>FOREVER BAMBU S.P.A. SOCIETA BENEFIT</t>
-        </is>
+      <c r="C6" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="D6" s="28"/>
       <c r="E6" s="18"/>
@@ -1753,10 +1751,8 @@
       <c r="B7" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>12072470961</t>
-        </is>
+      <c r="C7" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="D7" s="29"/>
       <c r="E7" s="18"/>
@@ -1793,10 +1789,8 @@
       <c r="B8" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Milano</t>
-        </is>
+      <c r="C8" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="18"/>
@@ -1880,26 +1874,12 @@
       <c r="B11" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>WP1 - Analisi dei processi, baseline KPI, requisiti, RACI e piano di test per Carbon Manager Learning Operations 4.0</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Sistemi di gestione dati aziendali (ERP, CRM, MES, DMS, HRMS, WMS, BI)</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>Italia Digitale S.r.l.</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>11914080962</t>
-        </is>
-      </c>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="9"/>
+      <c r="F11" s="10"/>
       <c r="G11" s="11">
         <v>8000</v>
       </c>
@@ -2009,26 +1989,12 @@
       <c r="B14" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>WP6 - Formazione del personale Forever Bambu su workflow operativi, dashboard, supervisione output AI, aggiornamento contenuti e procedure della piattaforma</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Intelligenza artificiale (Machine learning, Deep Learning, NLP, LLM, Agenti AI, data mining)</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>Italia Digitale S.r.l.</t>
-        </is>
-      </c>
-      <c r="F14" s="10" t="inlineStr">
-        <is>
-          <t>11914080962</t>
-        </is>
-      </c>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" s="9"/>
+      <c r="F14" s="10"/>
       <c r="G14" s="11">
         <v>5000</v>
       </c>
@@ -2138,26 +2104,12 @@
       <c r="B17" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Hosting Hetzner cloud/dedicated per integrazioni verticali e orizzontali, ambienti applicativi e test - 12 mesi</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>Cloud computing, Edge Computing</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>Italia Digitale S.r.l.</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="inlineStr">
-        <is>
-          <t>11914080962</t>
-        </is>
-      </c>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="9"/>
+      <c r="F17" s="10"/>
       <c r="G17" s="11">
         <v>2400</v>
       </c>
@@ -2190,26 +2142,12 @@
     </row>
     <row r="18" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B18" s="35"/>
-      <c r="C18" s="15" t="inlineStr">
-        <is>
-          <t>Database, backup, storage e monitoraggio dei servizi di progetto - 12 mesi</t>
-        </is>
-      </c>
-      <c r="D18" s="15" t="inlineStr">
-        <is>
-          <t>Cloud computing, Edge Computing</t>
-        </is>
-      </c>
-      <c r="E18" s="15" t="inlineStr">
-        <is>
-          <t>Italia Digitale S.r.l.</t>
-        </is>
-      </c>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>11914080962</t>
-        </is>
-      </c>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="E18" s="15"/>
+      <c r="F18" s="16"/>
       <c r="G18" s="17">
         <v>1800</v>
       </c>
@@ -2243,7 +2181,9 @@
     <row r="19" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B19" s="35"/>
       <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
+      <c r="D19" s="15" t="s">
+        <v>26</v>
+      </c>
       <c r="E19" s="15"/>
       <c r="F19" s="16"/>
       <c r="G19" s="17">
@@ -2279,7 +2219,9 @@
     <row r="20" spans="2:33" x14ac:dyDescent="0.25">
       <c r="B20" s="35"/>
       <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
+      <c r="D20" s="15" t="s">
+        <v>26</v>
+      </c>
       <c r="E20" s="15"/>
       <c r="F20" s="16"/>
       <c r="G20" s="17">
@@ -2355,26 +2297,12 @@
       <c r="B22" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>WP2 - Architettura, modello dati e integrazioni tra piattaforma corsi, survey/assessment, CRM, automazioni e dashboard; servizi di assessment, analytics e automazione dei flussi - 12 mesi</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Sistemi di gestione dati aziendali (ERP, CRM, MES, DMS, HRMS, WMS, BI)</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>Italia Digitale S.r.l.</t>
-        </is>
-      </c>
-      <c r="F22" s="10" t="inlineStr">
-        <is>
-          <t>11914080962</t>
-        </is>
-      </c>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="9"/>
+      <c r="F22" s="10"/>
       <c r="G22" s="11">
         <v>11200</v>
       </c>
@@ -2412,23 +2340,13 @@
           <t>WP3-WP5 - Sviluppo workflow AI human-in-the-loop, classificazione feedback e assessment, dashboard, pilota, test, collaudo e ottimizzazione della piattaforma Carbon Manager</t>
         </is>
       </c>
-      <c r="D23" s="15" t="inlineStr">
-        <is>
-          <t>Intelligenza artificiale (Machine learning, Deep Learning, NLP, LLM, Agenti AI, data mining)</t>
-        </is>
-      </c>
-      <c r="E23" s="15" t="inlineStr">
-        <is>
-          <t>Italia Digitale S.r.l.</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>11914080962</t>
-        </is>
-      </c>
+      <c r="D23" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="E23" s="15"/>
+      <c r="F23" s="16"/>
       <c r="G23" s="17">
-        <v>19600</v>
+        <v>25600</v>
       </c>
       <c r="H23" s="18"/>
       <c r="I23" s="18"/>
@@ -2622,7 +2540,7 @@
       <c r="E28" s="22"/>
       <c r="F28" s="22"/>
       <c r="G28" s="11">
-        <v>12000</v>
+        <v>6000</v>
       </c>
       <c r="H28" s="18"/>
       <c r="I28" s="20"/>
@@ -2737,10 +2655,8 @@
       <c r="D31" s="54"/>
       <c r="E31" s="54"/>
       <c r="F31" s="55"/>
-      <c r="G31" s="56" t="inlineStr">
-        <is>
-          <t>Seleziona opzione</t>
-        </is>
+      <c r="G31" s="56" t="s">
+        <v>47</v>
       </c>
       <c r="H31" s="18"/>
       <c r="I31" s="18"/>
@@ -2777,10 +2693,8 @@
       <c r="D32" s="54"/>
       <c r="E32" s="54"/>
       <c r="F32" s="55"/>
-      <c r="G32" s="56" t="inlineStr">
-        <is>
-          <t>Seleziona opzione</t>
-        </is>
+      <c r="G32" s="56" t="s">
+        <v>47</v>
       </c>
       <c r="H32" s="18"/>
       <c r="I32" s="18"/>

</xml_diff>